<commit_message>
updates indicators master spreadsheet for apprenticeship starts
</commit_message>
<xml_diff>
--- a/data/common_project_data/indicators-master.xlsx
+++ b/data/common_project_data/indicators-master.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\steve.crawshaw\projects\weca_regional_indicators\data\common_project_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FFDEA1C4-DE7A-4739-ACCF-6327D488E939}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AF6140F-7556-4554-B022-2CA80BDCCB8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-3510" windowWidth="16440" windowHeight="29040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="indicators" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1593" uniqueCount="829">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1593" uniqueCount="830">
   <si>
     <t>Unique ID</t>
   </si>
@@ -2565,6 +2565,9 @@
   </si>
   <si>
     <t>Weighted coverage</t>
+  </si>
+  <si>
+    <t>Starts</t>
   </si>
 </sst>
 </file>
@@ -6055,7 +6058,7 @@
         <v>1</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>105</v>
+        <v>829</v>
       </c>
       <c r="J39" s="1" t="s">
         <v>397</v>
@@ -15309,12 +15312,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d56b9130-d22a-480d-bb83-f34040f04d96">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Notes xmlns="d56b9130-d22a-480d-bb83-f34040f04d96" xsi:nil="true"/>
+    <TaxCatchAll xmlns="dd8606a3-d959-45f7-996e-3c98d970357c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -15587,21 +15593,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d56b9130-d22a-480d-bb83-f34040f04d96">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Notes xmlns="d56b9130-d22a-480d-bb83-f34040f04d96" xsi:nil="true"/>
-    <TaxCatchAll xmlns="dd8606a3-d959-45f7-996e-3c98d970357c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D4B7956-BCA0-46CA-BF6B-C7215DA15D81}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED897AD3-F0B7-437A-A46C-43145E78E644}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="d56b9130-d22a-480d-bb83-f34040f04d96"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="dd8606a3-d959-45f7-996e-3c98d970357c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -15626,18 +15638,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED897AD3-F0B7-437A-A46C-43145E78E644}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D4B7956-BCA0-46CA-BF6B-C7215DA15D81}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="d56b9130-d22a-480d-bb83-f34040f04d96"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="dd8606a3-d959-45f7-996e-3c98d970357c"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>